<commit_message>
[EXPERIMENTAL] Ramp up Faith weight
while ramp down religious units (much more useless than other civilians)
</commit_message>
<xml_diff>
--- a/文档/AI产出规划平衡.xlsx
+++ b/文档/AI产出规划平衡.xlsx
@@ -87,14 +87,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -567,133 +560,133 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -701,7 +694,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1443,11 +1436,11 @@
         <v>3</v>
       </c>
       <c r="G10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10">
         <f>SUM(B10:G10)</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J10">
         <f>B10-1</f>
@@ -1471,7 +1464,7 @@
       </c>
       <c r="O10">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1522,7 +1515,7 @@
       </c>
       <c r="O11">
         <f t="shared" si="14"/>
-        <v>-0.2</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="12" spans="1:15">

</xml_diff>

<commit_message>
ramp up early faith weight
</commit_message>
<xml_diff>
--- a/文档/AI产出规划平衡.xlsx
+++ b/文档/AI产出规划平衡.xlsx
@@ -1487,11 +1487,11 @@
         <v>1.3</v>
       </c>
       <c r="G11">
-        <v>0.8</v>
+        <v>1.3</v>
       </c>
       <c r="H11">
         <f t="shared" ref="H11:H15" si="13">SUM(B11:G11)</f>
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="J11">
         <f>B11-B10</f>
@@ -1515,7 +1515,7 @@
       </c>
       <c r="O11">
         <f t="shared" si="14"/>
-        <v>-1.2</v>
+        <v>-0.7</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="O12">
         <f t="shared" si="14"/>
-        <v>-0.3</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="13" spans="1:15">

</xml_diff>